<commit_message>
simulated D5 and D6 generated
</commit_message>
<xml_diff>
--- a/i_test/test_D6_Table_1/g_output/D6_Table_1_cohort_characteristics_GLP1RA.xlsx
+++ b/i_test/test_D6_Table_1/g_output/D6_Table_1_cohort_characteristics_GLP1RA.xlsx
@@ -518,47 +518,47 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>104</t>
+          <t>565</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>115</t>
+          <t>550</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>100</t>
+          <t>536</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>106</t>
+          <t>590</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>88</t>
+          <t>544</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>93</t>
+          <t>548</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>94</t>
+          <t>574</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>91</t>
+          <t>511</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>95</t>
+          <t>582</t>
         </is>
       </c>
     </row>
@@ -577,47 +577,47 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>49 (39.5 - 62.25)</t>
+          <t>50 (40 - 59)</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>53 (42.5 - 60.5)</t>
+          <t>50 (39 - 60)</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>49 (40 - 61)</t>
+          <t>50 (39 - 60)</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>47 (38 - 57.75)</t>
+          <t>51 (40 - 61.75)</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>52 (41.75 - 60)</t>
+          <t>51 (41 - 60.25)</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>51 (43 - 61)</t>
+          <t>50 (41 - 62)</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>53.5 (41.25 - 60.75)</t>
+          <t>50.5 (41 - 61)</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>53 (46 - 63.5)</t>
+          <t>50 (40 - 61)</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>47 (41 - 60.5)</t>
+          <t>51 (42 - 59)</t>
         </is>
       </c>
     </row>
@@ -636,47 +636,47 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>44 (42,3%)</t>
+          <t>195 (34,5%)</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>34 (29,6%)</t>
+          <t>201 (36,5%)</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>39 (39,0%)</t>
+          <t>194 (36,2%)</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>45 (42,5%)</t>
+          <t>203 (34,4%)</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>28 (31,8%)</t>
+          <t>187 (34,4%)</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>26 (28,0%)</t>
+          <t>195 (35,6%)</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>27 (28,7%)</t>
+          <t>188 (32,8%)</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>21 (23,1%)</t>
+          <t>182 (35,6%)</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>41 (43,2%)</t>
+          <t>182 (31,3%)</t>
         </is>
       </c>
     </row>
@@ -688,47 +688,47 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>38 (36,5%)</t>
+          <t>283 (50,1%)</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>63 (54,8%)</t>
+          <t>258 (46,9%)</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>46 (46,0%)</t>
+          <t>252 (47,0%)</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>47 (44,3%)</t>
+          <t>282 (47,8%)</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>51 (58,0%)</t>
+          <t>266 (48,9%)</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>50 (53,8%)</t>
+          <t>250 (45,6%)</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>48 (51,1%)</t>
+          <t>283 (49,3%)</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>50 (54,9%)</t>
+          <t>246 (48,1%)</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>34 (35,8%)</t>
+          <t>313 (53,8%)</t>
         </is>
       </c>
     </row>
@@ -740,47 +740,47 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>16 (15,4%)</t>
+          <t>64 (11,3%)</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>10 (8,7%)</t>
+          <t>64 (11,6%)</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>10 (10,0%)</t>
+          <t>65 (12,1%)</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>10 (9,4%)</t>
+          <t>74 (12,5%)</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>8 (9,1%)</t>
+          <t>70 (12,9%)</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>12 (12,9%)</t>
+          <t>75 (13,7%)</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>13 (13,8%)</t>
+          <t>66 (11,5%)</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>15 (16,5%)</t>
+          <t>54 (10,6%)</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>14 (14,7%)</t>
+          <t>62 (10,7%)</t>
         </is>
       </c>
     </row>
@@ -792,47 +792,47 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>6 (5,8%)</t>
+          <t>23 (4,1%)</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>8 (7,0%)</t>
+          <t>27 (4,9%)</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>5 (5,0%)</t>
+          <t>25 (4,7%)</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>4 (3,8%)</t>
+          <t>31 (5,3%)</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>1 (1,1%)</t>
+          <t>21 (3,9%)</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>5 (5,4%)</t>
+          <t>28 (5,1%)</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>6 (6,4%)</t>
+          <t>37 (6,4%)</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>5 (5,5%)</t>
+          <t>29 (5,7%)</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>6 (6,3%)</t>
+          <t>25 (4,3%)</t>
         </is>
       </c>
     </row>
@@ -844,47 +844,47 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>46 (44,2%)</t>
+          <t>291 (51,5%)</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>55 (47,8%)</t>
+          <t>289 (52,5%)</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>49 (49,0%)</t>
+          <t>284 (53,0%)</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>45 (42,5%)</t>
+          <t>282 (47,8%)</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>43 (48,9%)</t>
+          <t>254 (46,7%)</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>45 (48,4%)</t>
+          <t>271 (49,5%)</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>46 (48,9%)</t>
+          <t>282 (49,1%)</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>45 (49,5%)</t>
+          <t>242 (47,4%)</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>45 (47,4%)</t>
+          <t>298 (51,2%)</t>
         </is>
       </c>
     </row>
@@ -897,47 +897,47 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>74 (71,2%)</t>
+          <t>379 (67,1%)</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>82 (71,3%)</t>
+          <t>375 (68,2%)</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>61 (61,0%)</t>
+          <t>374 (69,8%)</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>71 (67,0%)</t>
+          <t>402 (68,1%)</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>63 (71,6%)</t>
+          <t>366 (67,3%)</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>59 (63,4%)</t>
+          <t>362 (66,1%)</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>64 (68,1%)</t>
+          <t>398 (69,3%)</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>55 (60,4%)</t>
+          <t>338 (66,1%)</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>71 (74,7%)</t>
+          <t>422 (72,5%)</t>
         </is>
       </c>
     </row>
@@ -950,47 +950,47 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>7 (6,7%)</t>
+          <t>49 (8,7%)</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>11 (9,6%)</t>
+          <t>38 (6,9%)</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>11 (11,0%)</t>
+          <t>42 (7,8%)</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>14 (13,2%)</t>
+          <t>54 (9,2%)</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>4 (4,5%)</t>
+          <t>44 (8,1%)</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>4 (4,3%)</t>
+          <t>48 (8,8%)</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>10 (10,6%)</t>
+          <t>58 (10,1%)</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>11 (12,1%)</t>
+          <t>44 (8,6%)</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>5 (5,3%)</t>
+          <t>45 (7,7%)</t>
         </is>
       </c>
     </row>
@@ -1009,47 +1009,47 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>43 (41,3%)</t>
+          <t>235 (41,6%)</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>43 (37,4%)</t>
+          <t>230 (41,8%)</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>42 (42,0%)</t>
+          <t>221 (41,2%)</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>42 (39,6%)</t>
+          <t>232 (39,3%)</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>34 (38,6%)</t>
+          <t>212 (39,0%)</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>35 (37,6%)</t>
+          <t>212 (38,7%)</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>35 (37,2%)</t>
+          <t>242 (42,2%)</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>33 (36,3%)</t>
+          <t>232 (45,4%)</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>45 (47,4%)</t>
+          <t>222 (38,1%)</t>
         </is>
       </c>
     </row>
@@ -1061,47 +1061,47 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>16 (15,4%)</t>
+          <t>96 (17,0%)</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>16 (13,9%)</t>
+          <t>82 (14,9%)</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>17 (17,0%)</t>
+          <t>72 (13,4%)</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>15 (14,2%)</t>
+          <t>82 (13,9%)</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>15 (17,0%)</t>
+          <t>76 (14,0%)</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>9 (9,7%)</t>
+          <t>67 (12,2%)</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>10 (10,6%)</t>
+          <t>89 (15,5%)</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>9 (9,9%)</t>
+          <t>71 (13,9%)</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>14 (14,7%)</t>
+          <t>77 (13,2%)</t>
         </is>
       </c>
     </row>
@@ -1113,47 +1113,47 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>85 (81,7%)</t>
+          <t>476 (84,2%)</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>92 (80,0%)</t>
+          <t>458 (83,3%)</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>87 (87,0%)</t>
+          <t>462 (86,2%)</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>96 (90,6%)</t>
+          <t>497 (84,2%)</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>78 (88,6%)</t>
+          <t>467 (85,8%)</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>75 (80,6%)</t>
+          <t>463 (84,5%)</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>80 (85,1%)</t>
+          <t>478 (83,3%)</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>76 (83,5%)</t>
+          <t>437 (85,5%)</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>81 (85,3%)</t>
+          <t>486 (83,5%)</t>
         </is>
       </c>
     </row>
@@ -1165,47 +1165,47 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>88 (84,6%)</t>
+          <t>483 (85,5%)</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>102 (88,7%)</t>
+          <t>472 (85,8%)</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>86 (86,0%)</t>
+          <t>454 (84,7%)</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>88 (83,0%)</t>
+          <t>503 (85,3%)</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>79 (89,8%)</t>
+          <t>460 (84,6%)</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>81 (87,1%)</t>
+          <t>464 (84,7%)</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>78 (83,0%)</t>
+          <t>488 (85,0%)</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>79 (86,8%)</t>
+          <t>424 (83,0%)</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>79 (83,2%)</t>
+          <t>492 (84,5%)</t>
         </is>
       </c>
     </row>
@@ -1217,47 +1217,47 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>58 (55,8%)</t>
+          <t>299 (52,9%)</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>51 (44,3%)</t>
+          <t>312 (56,7%)</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>49 (49,0%)</t>
+          <t>284 (53,0%)</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>56 (52,8%)</t>
+          <t>297 (50,3%)</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>43 (48,9%)</t>
+          <t>287 (52,8%)</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>53 (57,0%)</t>
+          <t>273 (49,8%)</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>47 (50,0%)</t>
+          <t>304 (53,0%)</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>44 (48,4%)</t>
+          <t>290 (56,8%)</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>50 (52,6%)</t>
+          <t>314 (54,0%)</t>
         </is>
       </c>
     </row>
@@ -1269,47 +1269,47 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>15 (14,4%)</t>
+          <t>118 (20,9%)</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>25 (21,7%)</t>
+          <t>109 (19,8%)</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>15 (15,0%)</t>
+          <t>100 (18,7%)</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>21 (19,8%)</t>
+          <t>105 (17,8%)</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>19 (21,6%)</t>
+          <t>105 (19,3%)</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>20 (21,5%)</t>
+          <t>94 (17,2%)</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>20 (21,3%)</t>
+          <t>114 (19,9%)</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>12 (13,2%)</t>
+          <t>88 (17,2%)</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>14 (14,7%)</t>
+          <t>96 (16,5%)</t>
         </is>
       </c>
     </row>

</xml_diff>